<commit_message>
[200~feat: implementa extrator de autos via Gemini File API
Corpo:

    Adiciona leitor_processos.py para automatizar a leitura de PDFs de processos judiciais e preenchimento de template.

    Implementa upload via File API do Gemini, permitindo processamento de arquivos grandes sem estouro de limite de texto.

    Adiciona .env para gerenciamento seguro de credenciais (adicionado ao .gitignore).

    Inclui tratamento de erros e interface gráfica via Tkinter para suporte ao fluxo de trabalho jurídico.
</commit_message>
<xml_diff>
--- a/Processos_Entrada/template_nash.xlsx
+++ b/Processos_Entrada/template_nash.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Danos" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Custas" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Deducoes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t xml:space="preserve">Processo</t>
   </si>
   <si>
-    <t xml:space="preserve">5006562-94.2024.8.13.0313</t>
+    <t xml:space="preserve">5064418-49.2020.8.13.0024</t>
   </si>
   <si>
     <t xml:space="preserve">Data do Trânsito</t>
@@ -36,7 +37,10 @@
     <t xml:space="preserve">Data da Sentença</t>
   </si>
   <si>
-    <t xml:space="preserve">Termo inicial Juros</t>
+    <t xml:space="preserve">Termo Inicial Juros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desembolso</t>
   </si>
   <si>
     <t xml:space="preserve">Data da Citação</t>
@@ -48,7 +52,13 @@
     <t xml:space="preserve">Justiça Gratuita</t>
   </si>
   <si>
-    <t xml:space="preserve">Não</t>
+    <t xml:space="preserve">não</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fazenda Pública</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sim</t>
   </si>
   <si>
     <t xml:space="preserve">Pagamento Voluntário 15d</t>
@@ -75,40 +85,82 @@
     <t xml:space="preserve">Regra</t>
   </si>
   <si>
-    <t xml:space="preserve">Evento 1, DOCCOMPROV7, Página 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023/230</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID 10198424660, pág. 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pagamento indenização int</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evento 5, TRASLADO2, Página 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Custas iniciais </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evento 41, DOCCOMPROV2, Página 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Int testemunha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evento 41, DOCCOMPROV3, Página 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evento 41, DOCCOMPROV4, Página 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evento 42, DOCCOMPROV2, Página 1</t>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV13, Página 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0000.82624</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV13, Página 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000.000.120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV13, Página 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0000.82836</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV13, Página 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000.011.424</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV13, Página 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000.000.670</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV13, Página 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">000.000.253</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 1, DOCCOMPROV12, Página 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 4, TRASLADO3, Página 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custas iniciais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 20, TRASLADO3, Página 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citação O.J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 84, TRASLADO4, Página 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SISBAJUD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 84, TRASLADO6, Página 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RENAJUD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evento 109, TRASLADO4, Página 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alvara </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data bloqueio/deposito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
   </si>
 </sst>
 </file>
@@ -321,11 +373,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.32"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -340,58 +392,75 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2" t="n">
+        <v>45404</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45989</v>
+        <v>45192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>43334</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -410,7 +479,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.08"/>
@@ -422,66 +491,154 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45125</v>
+        <v>43178</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>173.63</v>
+        <v>270.97</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45120</v>
+        <v>43180</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>16160</v>
+        <v>500</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="2"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>43181</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>55.93</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>43186</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>43190</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>350</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>43229</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>390</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>1863</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>43243</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>377.77</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -510,107 +667,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45383</v>
+        <v>43997</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>655.74</v>
+        <v>429.84</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45736</v>
+        <v>44274</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>18.05</v>
+        <v>25.24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45736</v>
+        <v>45797</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>18.05</v>
+        <v>13.27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45736</v>
+        <v>45797</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>18.05</v>
+        <v>13.27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45761</v>
+        <v>45889</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>18.05</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>66.37</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C13" s="2"/>
     </row>
   </sheetData>
@@ -622,4 +779,38 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.79"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2"/>
+      <c r="B2" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPágina &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>